<commit_message>
working but 14 bin
</commit_message>
<xml_diff>
--- a/SLF_Modul_Metodolojileri.xlsx
+++ b/SLF_Modul_Metodolojileri.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emre Hangul\Desktop\MRC\SLF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96479E72-09AB-4B48-9A93-B2D97BD39910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97E6891D-AD24-408F-B100-097EB4CC8AA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,27 @@
     <sheet name="Notlar ve Bilinen Riskler" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metodoloji!$A$2:$H$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metodoloji!$A$2:$H$45</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="247">
   <si>
     <t>SLF (Spatial Load Forecasting) — Modül Metodolojileri</t>
   </si>
@@ -218,42 +231,12 @@
     <t>Overpass API/CSV, KML zonlama planı poligonları</t>
   </si>
   <si>
-    <t>KML dosyasındaki poligonlar bir coğrafi veri tablosuna aktarılır (nokta-yük poligonları ayrıca ayrıştırılır); bu tablo, OpenStreetMap'ten gelen bina/parsel verisiyle mekânsal olarak kesiştirilip katman tipine göre ayrılır.</t>
-  </si>
-  <si>
     <t>İMAR_SONUÇLAR (CSV/KML/SHP), parsel-kesişim tablosu</t>
   </si>
   <si>
     <t>Kod/imar/python_kod/imar_analizi/main.py, imar_check.py, imar_datalar.py</t>
   </si>
   <si>
-    <t>Adım 2: 3 kademeli nokta-bina eşleştirme</t>
-  </si>
-  <si>
-    <t>Abone noktaları (mesken/ticarethane), bina poligonları, parsel sınırları</t>
-  </si>
-  <si>
-    <t>Kademe 1: nokta doğrudan bir bina poligonunun içindeyse eşleşir. Kademe 2: eşleşmeyen noktalar için binalar yaklaşık 20 metre genişletilir, bu genişletilmiş alana düşen noktalar, en yakın bina merkezine eşleştirilir. Kademe 3: hâlâ eşleşmeyen noktalarda, noktanın kendisi yaklaşık 10 metre genişletilir ve içinde bulunduğu parselin ortalama bina büyüklüğünden bir alan tahmini yapılır.</t>
-  </si>
-  <si>
-    <t>Nokta-bina eşleşme tablosu (TAKS/KAKS/yükseklik dahil)</t>
-  </si>
-  <si>
-    <t>Kod/imar/python_kod/imar_analizi/kod/kofre_analiz/imar_tipleri_analizi_v2.py</t>
-  </si>
-  <si>
-    <t>Adım 3: Bina tipi istatistik tabloları</t>
-  </si>
-  <si>
-    <t>Eşleşmiş nokta-bina verisi</t>
-  </si>
-  <si>
-    <t>Bina kat grubu (1-2/3-4/5-7/8+ katlı/villa mesken) ve bina tipi (küçük/orta/büyük sanayi-ticarethane) bazında ortalama TAKS, bina alanı, yükseklik ve metrekare/abone başına tüketim hesaplanır.</t>
-  </si>
-  <si>
-    <t>mesken_istatistikleri.csv, ticaret_istatistikleri.csv (doluluk oranı modelinin girdisi)</t>
-  </si>
-  <si>
     <t>Yapay zeka ile bina alt-tipi (kat sayısı) tahmini</t>
   </si>
   <si>
@@ -263,27 +246,12 @@
     <t>Ham abone verisi (abone grubu, bağlantı gücü, yıllık tüketim)</t>
   </si>
   <si>
-    <t>Farklı yazım biçimleriyle girilmiş abone grubu adları (Türkçe karakter varyasyonları dahil) altı standart kategoriye — Mesken, Ticarethane, Sanayi, Tarımsal Sulama, Aydınlatma, Üretici — indirgenir ve bina bazında toplulaştırılır. Bir binadaki abonelerin %70'inden fazlası mesken ise bina 'Mesken' olarak etiketlenir; değilse bağlantı gücü ve tüketim miktarına göre (örneğin 150 kW ve 300.000 kWh üzerindeki tesisler 'Büyük Sanayi') alt tiplere ayrılır.</t>
-  </si>
-  <si>
     <t>Bina bazlı standart tip etiketi</t>
   </si>
   <si>
     <t>Kod/imar/python_kod/deep_learning/kod/model_learning.py</t>
   </si>
   <si>
-    <t>Adım 2: Makine öğrenmesi modeli ile kat-sayısı tahmini</t>
-  </si>
-  <si>
-    <t>3 özellik: ortalama mesken tüketimi, ortalama bağlantı gücü, mesken abone sayısı</t>
-  </si>
-  <si>
-    <t>Bu üç özellik standart bir ölçeklendirmeden geçirilir, verinin %80'i eğitim, %20'si test için ayrılır. Bir gradyan artırmalı ağaç modeli (XGBoost, varsayılan ayarlarla) eğitilip her bina için 1 ile 5 arası bir kat-sayısı sınıfı tahmin edilir. Eğitim verisi veya gerekli kolonlar eksikse, bina doğrudan '5-7 katlı' sınıfına (sabit varsayılan) atanır.</t>
-  </si>
-  <si>
-    <t>Bina bazlı kat-sayısı/tip tahmini + kayıtlı model dosyası</t>
-  </si>
-  <si>
     <t>Satürasyon (arazi doluluk oranı) modeli</t>
   </si>
   <si>
@@ -293,39 +261,12 @@
     <t>Uydu bazlı yapılaşma oranı, hücre bazlı bina/imar kırılımları</t>
   </si>
   <si>
-    <t>Uydu görüntülerinden gelen ham yapılaşma oranı önce gürültüden arındırılır: %5'in altındaki değerler sıfıra, %35'in üzerindeki değerler ise tamamen doymuş kabul edilip bire yuvarlanır. Ardından hücredeki 11 farklı bina alt-tipinin bina sayılarıyla ağırlıklandırılmış ortalama TAKS değeri hesaplanır.</t>
-  </si>
-  <si>
     <t>Hücre bazlı ağırlıklı TAKS ve filtrelenmiş yapılaşma oranı</t>
   </si>
   <si>
     <t>Kod/imar/python_kod/imar_analizi/kod/saturasyon/saturasyon_analiz.py</t>
   </si>
   <si>
-    <t>Adım 2: Net yapılabilir alan ve gerçek kullanım oranı</t>
-  </si>
-  <si>
-    <t>İmar alanı toplamı, ağırlıklı TAKS, hücre alanı</t>
-  </si>
-  <si>
-    <t>Hücrenin yapı yasağı olmayan imarlı alanından sabit bir %20'lik yol/kaldırım payı düşülür, kalan alan ağırlıklı TAKS değeriyle çarpılarak net yapılabilir alan bulunur. Gerçek kullanım oranı ise, hücredeki toplam bina alanının bu yapı-izinli alana oranı olarak hesaplanır (oran 1'i geçemez).</t>
-  </si>
-  <si>
-    <t>Hücre bazlı net alan ve kullanım oranları</t>
-  </si>
-  <si>
-    <t>Adım 3: Doluluk sınıflandırması ve nihai oran</t>
-  </si>
-  <si>
-    <t>Yapılaşma oranı, net yapılabilir/yapılı alan</t>
-  </si>
-  <si>
-    <t>Her hücre önce dört durumdan birine sınıflandırılır: imarlı/imarsız yeni genişleme bölgesi, kentsel yerleşim alanı veya kent dışı alan. Yapılı alan, hesaplanan net yapılabilir alanı aşıyorsa doluluk oranı doğrudan %100 kabul edilir. Uydu görüntüsünden hesaplanan oran ile bina sayımından hesaplanan oran arasında %20'den fazla fark varsa, bina sayımına dayalı (daha güvenilir kabul edilen) oran esas alınır.</t>
-  </si>
-  <si>
-    <t>Hücre × yıl bazlı doluluk oranı (0-1 arası) — Uzamsal Yük Tahmini modülünün girdisi</t>
-  </si>
-  <si>
     <t>İmar oranı (zonlama karışımı) çok-yıllı ileri projeksiyonu</t>
   </si>
   <si>
@@ -335,37 +276,10 @@
     <t>Doluluk oranı sıfırın üzerinde olan hücreler</t>
   </si>
   <si>
-    <t>Bu hücreler, birbirine yakınlıklarına göre (yaklaşık 500 metre içinde olanlar) gruplara ayrılır; 1000'den fazla hücre içeren büyük gruplar yaklaşık 50'şer hücrelik alt gruplara bölünür. Henüz doluluk oranı olmayan yeni genişleme hücrelerine, komşu kentsel hücrelerin ortalama doluluk oranı aktarılır; hücre imarsızsa bu değer yarıya düşürülerek uygulanır.</t>
-  </si>
-  <si>
     <t>Genişletilmiş doluluk oranı haritası (yıl bazlı)</t>
   </si>
   <si>
     <t>Kod/SLF/imar_oranı_tahmini.py</t>
-  </si>
-  <si>
-    <t>Adım 2: Yıllık organik büyüme eklenmesi</t>
-  </si>
-  <si>
-    <t>Uygun hücreler (en fazla 500)</t>
-  </si>
-  <si>
-    <t>Uygun hücrelere her yıl, %5 ile %15 arasında rastgele seçilen bir doluluk-oranı artışı eklenir (üst sınır %100); bu, doğal yıllık yoğunlaşmayı simüle eder. Komşu hücrelerin aranma yarıçapı, tahmin ufku ilerledikçe 200 metreden 280 metreye kademeli olarak genişler.</t>
-  </si>
-  <si>
-    <t>Yıl bazlı güncellenmiş doluluk oranı değerleri</t>
-  </si>
-  <si>
-    <t>Adım 3: Komşuluk bazlı zonlama karışımı tahmini</t>
-  </si>
-  <si>
-    <t>Büyüyen hücreler ve 500 metre içindeki komşuları</t>
-  </si>
-  <si>
-    <t>Gelişmiş (doluluk oranı yüksek) komşu hücrelerin imar tipi karışımı — örneğin mesken/sanayi/ticarethane payları — yeni büyüyen hücrelere mesafeye göre ağırlıklandırılarak aktarılır: yakın ve doluluk oranı yüksek komşuların etkisi daha fazladır. Böylece henüz gelişmemiş bir hücre için, çevresindeki gelişmiş hücrelere benzer bir imar karışımı tahmin edilmiş olur.</t>
-  </si>
-  <si>
-    <t>Yıl bazlı hücre zonlama karışımı tablosu (Abone Sayısı Tahmini modülünün girdisi)</t>
   </si>
   <si>
     <t>DEK (Dağıtık Enerji Kaynakları) Modülü</t>
@@ -1027,6 +941,228 @@
         <rFont val="Arial"/>
       </rPr>
       <t>Regresyon modeliyle zaman serisi modelinin tahmin hataları karşılaştırılır, hangisi daha isabetliyse o seçilir (Tarımsal Sulama segmentinde her zaman regresyon modeli kullanılır). Tahminler yıl yıl ileriye doğru üretilir: bir yılın tahmini, bir sonraki yılın hesaplamasında girdi olarak kullanılır.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t xml:space="preserve"> KML dosyasındaki poligonlar bir coğrafi veri tablosuna aktarılır (nokta-yük poligonları ayrıca ayrıştırılır); bu tablo, OpenStreetMap'ten gelen bina/parsel verisiyle mekânsal olarak kesiştirilip katman tipine göre ayrılır.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t xml:space="preserve"> Kademe 1: nokta doğrudan bir bina poligonunun içindeyse eşleşir. Kademe 2: eşleşmeyen noktalar için binalar yaklaşık 20 metre genişletilir, bu genişletilmiş alana düşen noktalar, en yakın bina merkezine eşleştirilir. Kademe 3: hâlâ eşleşmeyen noktalarda, noktanın kendisi yaklaşık 10 metre genişletilir ve içinde bulunduğu parselin ortalama bina büyüklüğünden bir alan tahmini yapılır.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t xml:space="preserve"> Bina kat grubu (1-2/3-4/5-7/8+ katlı/villa mesken) ve bina tipi (küçük/orta/büyük sanayi-ticarethane) bazında ortalama TAKS, bina alanı, yükseklik ve metrekare/abone başına tüketim hesaplanır.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t xml:space="preserve"> Farklı yazım biçimleriyle girilmiş abone grubu adları (Türkçe karakter varyasyonları dahil) altı standart kategoriye — Mesken, Ticarethane, Sanayi, Tarımsal Sulama, Aydınlatma, Üretici — indirgenir ve bina bazında toplulaştırılır. Bir binadaki abonelerin %70'inden fazlası mesken ise bina 'Mesken' olarak etiketlenir; değilse bağlantı gücü ve tüketim miktarına göre (örneğin 150 kW ve 300.000 kWh üzerindeki tesisler 'Büyük Sanayi') alt tiplere ayrılır.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t xml:space="preserve"> Bu üç özellik standart bir ölçeklendirmeden geçirilir, verinin %80'i eğitim, %20'si test için ayrılır. Bir gradyan artırmalı ağaç modeli (XGBoost, varsayılan ayarlarla) eğitilip her bina için 1 ile 5 arası bir kat-sayısı sınıfı tahmin edilir. Eğitim verisi veya gerekli kolonlar eksikse, bina doğrudan '5-7 katlı' sınıfına (sabit varsayılan) atanır.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t xml:space="preserve"> Uydu görüntülerinden gelen ham yapılaşma oranı önce gürültüden arındırılır: %5'in altındaki değerler sıfıra, %35'in üzerindeki değerler ise tamamen doymuş kabul edilip bire yuvarlanır. Ardından hücredeki 11 farklı bina alt-tipinin bina sayılarıyla ağırlıklandırılmış ortalama TAKS değeri hesaplanır.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t xml:space="preserve"> Hücrenin yapı yasağı olmayan imarlı alanından sabit bir %20'lik yol/kaldırım payı düşülür, kalan alan ağırlıklı TAKS değeriyle çarpılarak net yapılabilir alan bulunur. Gerçek kullanım oranı ise, hücredeki toplam bina alanının bu yapı-izinli alana oranı olarak hesaplanır (oran 1'i geçemez).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t xml:space="preserve"> Her hücre önce dört durumdan birine sınıflandırılır: imarlı/imarsız yeni genişleme bölgesi, kentsel yerleşim alanı veya kent dışı alan. Yapılı alan, hesaplanan net yapılabilir alanı aşıyorsa doluluk oranı doğrudan %100 kabul edilir. Uydu görüntüsünden hesaplanan oran ile bina sayımından hesaplanan oran arasında %20'den fazla fark varsa, bina sayımına dayalı (daha güvenilir kabul edilen) oran esas alınır.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve"> Bu hücreler, birbirine yakınlıklarına göre (yaklaşık 500 metre içinde olanlar) gruplara ayrılır; 1000'den fazla hücre içeren büyük gruplar yaklaşık 50'şer hücrelik alt gruplara bölünür. Henüz doluluk oranı olmayan yeni genişleme hücrelerine, komşu kentsel hücrelerin ortalama doluluk oranı aktarılır; hücre imarsızsa bu değer yarıya düşürülerek uygulanır.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve"> Uygun hücrelere her yıl, %5 ile %15 arasında rastgele seçilen bir doluluk-oranı artışı eklenir (üst sınır %100); bu, doğal yıllık yoğunlaşmayı simüle eder. Komşu hücrelerin aranma yarıçapı, tahmin ufku ilerledikçe 200 metreden 280 metreye kademeli olarak genişler.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="162"/>
+      </rPr>
+      <t xml:space="preserve"> Gelişmiş (doluluk oranı yüksek) komşu hücrelerin imar tipi karışımı — örneğin mesken/sanayi/ticarethane payları — yeni büyüyen hücrelere mesafeye göre ağırlıklandırılarak aktarılır: yakın ve doluluk oranı yüksek komşuların etkisi daha fazladır. Böylece henüz gelişmemiş bir hücre için, çevresindeki gelişmiş hücrelere benzer bir imar karışımı tahmin edilmiş olur.</t>
     </r>
   </si>
 </sst>
@@ -1154,7 +1290,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1219,6 +1355,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1523,7 +1662,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.109375" style="18" customWidth="1"/>
@@ -1591,7 +1730,7 @@
         <v>12</v>
       </c>
       <c r="F3" s="23" t="s">
-        <v>274</v>
+        <v>241</v>
       </c>
       <c r="G3" s="12" t="s">
         <v>13</v>
@@ -1617,7 +1756,7 @@
         <v>18</v>
       </c>
       <c r="F4" s="23" t="s">
-        <v>273</v>
+        <v>240</v>
       </c>
       <c r="G4" s="12" t="s">
         <v>19</v>
@@ -1643,7 +1782,7 @@
         <v>24</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>275</v>
+        <v>242</v>
       </c>
       <c r="G5" s="12" t="s">
         <v>25</v>
@@ -1669,7 +1808,7 @@
         <v>28</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>272</v>
+        <v>239</v>
       </c>
       <c r="G6" s="12" t="s">
         <v>29</v>
@@ -1678,457 +1817,457 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="20" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="13">
+    <row r="7" spans="1:8" s="20" customFormat="1" ht="139.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="14">
+        <v>20</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="F7" s="24" t="s">
+        <v>243</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="20" customFormat="1" ht="132" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="14">
+        <v>23</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>244</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="20" customFormat="1" ht="177" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="14">
+        <v>25</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="F9" s="24" t="s">
+        <v>245</v>
+      </c>
+      <c r="G9" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" s="20" customFormat="1" ht="170.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="14">
+        <v>28</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="F10" s="24" t="s">
+        <v>246</v>
+      </c>
+      <c r="G10" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="20" customFormat="1" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="13">
         <v>14</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="13">
-        <v>15</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="F8" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="G8" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" s="20" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="13">
-        <v>16</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="G9" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="13">
-        <v>17</v>
-      </c>
-      <c r="B10" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="F10" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="G10" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="13">
-        <v>18</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>31</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" s="20" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A12" s="13">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B12" s="13" t="s">
         <v>31</v>
       </c>
       <c r="C12" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="G12" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" s="20" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A13" s="13">
+        <v>16</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="13">
+        <v>17</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D14" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="G14" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="13">
+        <v>18</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="G15" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" s="20" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="13">
+        <v>19</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E16" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F16" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="G12" s="13" t="s">
+      <c r="G16" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="H16" s="3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="14">
-        <v>20</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="D13" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="F13" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="G13" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" s="20" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="14">
-        <v>21</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="F14" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="G14" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="14">
-        <v>22</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C15" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="D15" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="E15" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="F15" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="G15" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" s="20" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="14">
-        <v>23</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="F16" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="G16" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="H16" s="4" t="s">
+    <row r="17" spans="1:8" s="20" customFormat="1" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="15">
+        <v>31</v>
+      </c>
+      <c r="B17" s="15" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="14">
-        <v>24</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="D17" s="14" t="s">
+      <c r="C17" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="E17" s="14" t="s">
+      <c r="D17" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="F17" s="14" t="s">
+      <c r="E17" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="G17" s="14" t="s">
+      <c r="F17" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="H17" s="4" t="s">
+      <c r="G17" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" s="20" customFormat="1" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="15">
+        <v>32</v>
+      </c>
+      <c r="B18" s="15" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="14">
-        <v>25</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="E18" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="F18" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="G18" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="H18" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="D18" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="F18" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="G18" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="H18" s="4" t="s">
+    </row>
+    <row r="19" spans="1:8" s="20" customFormat="1" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="15">
+        <v>33</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C19" s="15" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="14">
-        <v>26</v>
-      </c>
-      <c r="B19" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="D19" s="14" t="s">
+      <c r="D19" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="E19" s="14" t="s">
+      <c r="E19" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="F19" s="14" t="s">
+      <c r="F19" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="G19" s="14" t="s">
+      <c r="G19" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="H19" s="4" t="s">
+      <c r="H19" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" s="20" customFormat="1" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="15">
+        <v>34</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="15" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" s="20" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="14">
-        <v>27</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="D20" s="14" t="s">
+      <c r="D20" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="F20" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="G20" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="H20" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="E20" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="F20" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="G20" s="14" t="s">
-        <v>99</v>
-      </c>
-      <c r="H20" s="4" t="s">
+    </row>
+    <row r="21" spans="1:8" s="20" customFormat="1" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="15">
+        <v>35</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C21" s="15" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="14">
-        <v>28</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="D21" s="14" t="s">
+      <c r="D21" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="E21" s="14" t="s">
+      <c r="E21" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="F21" s="14" t="s">
+      <c r="F21" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="G21" s="14" t="s">
+      <c r="G21" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="H21" s="4" t="s">
+      <c r="H21" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" s="20" customFormat="1" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="15">
+        <v>36</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C22" s="15" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="14">
-        <v>29</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="D22" s="14" t="s">
+      <c r="D22" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="E22" s="14" t="s">
+      <c r="E22" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="F22" s="14" t="s">
+      <c r="F22" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="G22" s="14" t="s">
+      <c r="G22" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="H22" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" s="20" customFormat="1" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="15">
+        <v>37</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C23" s="15" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="14">
-        <v>30</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="D23" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="E23" s="14" t="s">
+      <c r="D23" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="F23" s="14" t="s">
+      <c r="E23" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="G23" s="14" t="s">
+      <c r="F23" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="H23" s="4" t="s">
+      <c r="G23" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" s="20" customFormat="1" ht="62.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="15">
+        <v>38</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C24" s="15" t="s">
         <v>105</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="15">
-        <v>31</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="C24" s="15" t="s">
-        <v>115</v>
       </c>
       <c r="D24" s="15" t="s">
         <v>116</v>
@@ -2140,742 +2279,560 @@
         <v>118</v>
       </c>
       <c r="G24" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" s="20" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="16">
+        <v>39</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="D25" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="E25" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="F25" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="G25" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="H24" s="5" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" s="20" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="15">
-        <v>32</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="C25" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="D25" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="E25" s="15" t="s">
+      <c r="H25" s="6" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" s="20" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="16">
+        <v>40</v>
+      </c>
+      <c r="B26" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="F25" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="G25" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="H25" s="5" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" s="20" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="15">
-        <v>33</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="C26" s="15" t="s">
+      <c r="C26" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="D26" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="E26" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="F26" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="G26" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="H26" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="D26" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="E26" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="F26" s="15" t="s">
+    </row>
+    <row r="27" spans="1:8" s="20" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="16">
+        <v>41</v>
+      </c>
+      <c r="B27" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="C27" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="G26" s="15" t="s">
+      <c r="D27" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="H26" s="5" t="s">
+      <c r="E27" s="16" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="15">
-        <v>34</v>
-      </c>
-      <c r="B27" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="C27" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="D27" s="15" t="s">
+      <c r="F27" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="E27" s="15" t="s">
+      <c r="G27" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="F27" s="15" t="s">
+      <c r="H27" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="G27" s="15" t="s">
+    </row>
+    <row r="28" spans="1:8" s="20" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="16">
+        <v>42</v>
+      </c>
+      <c r="B28" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="D28" s="16" t="s">
         <v>133</v>
       </c>
-      <c r="H27" s="5" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" s="20" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A28" s="15">
-        <v>35</v>
-      </c>
-      <c r="B28" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="D28" s="15" t="s">
+      <c r="E28" s="16" t="s">
         <v>134</v>
       </c>
-      <c r="E28" s="15" t="s">
+      <c r="F28" s="16" t="s">
         <v>135</v>
       </c>
-      <c r="F28" s="15" t="s">
+      <c r="G28" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="G28" s="15" t="s">
+      <c r="H28" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" s="20" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="16">
+        <v>43</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="C29" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="H28" s="5" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" s="20" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A29" s="15">
-        <v>36</v>
-      </c>
-      <c r="B29" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="C29" s="15" t="s">
+      <c r="D29" s="16" t="s">
         <v>138</v>
       </c>
-      <c r="D29" s="15" t="s">
+      <c r="E29" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="E29" s="15" t="s">
+      <c r="F29" s="16" t="s">
         <v>140</v>
       </c>
-      <c r="F29" s="15" t="s">
+      <c r="G29" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="G29" s="15" t="s">
+      <c r="H29" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" s="20" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="16">
+        <v>44</v>
+      </c>
+      <c r="B30" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="D30" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="H29" s="5" t="s">
+      <c r="E30" s="16" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="15">
-        <v>37</v>
-      </c>
-      <c r="B30" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="C30" s="15" t="s">
-        <v>138</v>
-      </c>
-      <c r="D30" s="15" t="s">
+      <c r="F30" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="E30" s="15" t="s">
+      <c r="G30" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="F30" s="15" t="s">
+      <c r="H30" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" s="20" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="16">
+        <v>45</v>
+      </c>
+      <c r="B31" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="D31" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="G30" s="15" t="s">
+      <c r="E31" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="H30" s="5" t="s">
+      <c r="F31" s="16" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" s="20" customFormat="1" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A31" s="15">
-        <v>38</v>
-      </c>
-      <c r="B31" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>138</v>
-      </c>
-      <c r="D31" s="15" t="s">
+      <c r="G31" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="E31" s="15" t="s">
+      <c r="H31" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" s="20" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="16">
+        <v>46</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="C32" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="F31" s="15" t="s">
+      <c r="D32" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="G31" s="15" t="s">
+      <c r="E32" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="H31" s="5" t="s">
+      <c r="F32" s="16" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" s="20" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A32" s="16">
-        <v>39</v>
-      </c>
-      <c r="B32" s="16" t="s">
+      <c r="G32" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="C32" s="16" t="s">
-        <v>115</v>
-      </c>
-      <c r="D32" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="E32" s="16" t="s">
+      <c r="H32" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" s="20" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="16">
+        <v>47</v>
+      </c>
+      <c r="B33" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="D33" s="16" t="s">
         <v>155</v>
       </c>
-      <c r="F32" s="16" t="s">
+      <c r="E33" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="G32" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="H32" s="6" t="s">
+      <c r="F33" s="16" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" s="20" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A33" s="16">
-        <v>40</v>
-      </c>
-      <c r="B33" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="C33" s="16" t="s">
-        <v>115</v>
-      </c>
-      <c r="D33" s="16" t="s">
-        <v>120</v>
-      </c>
-      <c r="E33" s="16" t="s">
+      <c r="G33" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" s="20" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="16">
+        <v>48</v>
+      </c>
+      <c r="B34" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="F33" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="G33" s="16" t="s">
+      <c r="C34" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="H33" s="6" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="16">
-        <v>41</v>
-      </c>
-      <c r="B34" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="C34" s="16" t="s">
+      <c r="D34" s="16" t="s">
         <v>160</v>
       </c>
-      <c r="D34" s="16" t="s">
+      <c r="E34" s="16" t="s">
         <v>161</v>
       </c>
-      <c r="E34" s="16" t="s">
+      <c r="F34" s="16" t="s">
         <v>162</v>
       </c>
-      <c r="F34" s="16" t="s">
+      <c r="G34" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="G34" s="16" t="s">
+      <c r="H34" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" s="20" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="16">
+        <v>49</v>
+      </c>
+      <c r="B35" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="D35" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="H34" s="6" t="s">
+      <c r="E35" s="16" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" s="20" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A35" s="16">
-        <v>42</v>
-      </c>
-      <c r="B35" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="C35" s="16" t="s">
-        <v>160</v>
-      </c>
-      <c r="D35" s="16" t="s">
+      <c r="F35" s="16" t="s">
         <v>166</v>
       </c>
-      <c r="E35" s="16" t="s">
+      <c r="G35" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="F35" s="16" t="s">
+      <c r="H35" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" s="20" customFormat="1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="16">
+        <v>50</v>
+      </c>
+      <c r="B36" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="D36" s="16" t="s">
         <v>168</v>
       </c>
-      <c r="G35" s="16" t="s">
+      <c r="E36" s="16" t="s">
         <v>169</v>
       </c>
-      <c r="H35" s="6" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" s="20" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A36" s="16">
-        <v>43</v>
-      </c>
-      <c r="B36" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="C36" s="16" t="s">
+      <c r="F36" s="16" t="s">
         <v>170</v>
       </c>
-      <c r="D36" s="16" t="s">
+      <c r="G36" s="16" t="s">
         <v>171</v>
       </c>
-      <c r="E36" s="16" t="s">
+      <c r="H36" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" s="20" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A37" s="17">
+        <v>51</v>
+      </c>
+      <c r="B37" s="17" t="s">
         <v>172</v>
       </c>
-      <c r="F36" s="16" t="s">
+      <c r="C37" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="G36" s="16" t="s">
+      <c r="D37" s="17" t="s">
         <v>174</v>
       </c>
-      <c r="H36" s="6" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A37" s="16">
-        <v>44</v>
-      </c>
-      <c r="B37" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="C37" s="16" t="s">
-        <v>170</v>
-      </c>
-      <c r="D37" s="16" t="s">
+      <c r="E37" s="17" t="s">
         <v>175</v>
       </c>
-      <c r="E37" s="16" t="s">
+      <c r="F37" s="17" t="s">
         <v>176</v>
       </c>
-      <c r="F37" s="16" t="s">
+      <c r="G37" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="G37" s="16" t="s">
+      <c r="H37" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="H37" s="6" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" s="20" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A38" s="16">
-        <v>45</v>
-      </c>
-      <c r="B38" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="C38" s="16" t="s">
-        <v>170</v>
-      </c>
-      <c r="D38" s="16" t="s">
+    </row>
+    <row r="38" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A38" s="17">
+        <v>52</v>
+      </c>
+      <c r="B38" s="17" t="s">
+        <v>172</v>
+      </c>
+      <c r="C38" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="D38" s="17" t="s">
         <v>179</v>
       </c>
-      <c r="E38" s="16" t="s">
+      <c r="E38" s="17" t="s">
         <v>180</v>
       </c>
-      <c r="F38" s="16" t="s">
+      <c r="F38" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="G38" s="16" t="s">
+      <c r="G38" s="17" t="s">
         <v>182</v>
       </c>
-      <c r="H38" s="6" t="s">
-        <v>165</v>
+      <c r="H38" s="7" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="39" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A39" s="16">
-        <v>46</v>
-      </c>
-      <c r="B39" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="C39" s="16" t="s">
+      <c r="A39" s="17">
+        <v>53</v>
+      </c>
+      <c r="B39" s="17" t="s">
+        <v>172</v>
+      </c>
+      <c r="C39" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="D39" s="17" t="s">
+        <v>184</v>
+      </c>
+      <c r="E39" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="F39" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="G39" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="17">
+        <v>54</v>
+      </c>
+      <c r="B40" s="17" t="s">
+        <v>172</v>
+      </c>
+      <c r="C40" s="17" t="s">
+        <v>189</v>
+      </c>
+      <c r="D40" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="E40" s="17" t="s">
+        <v>191</v>
+      </c>
+      <c r="F40" s="17" t="s">
+        <v>192</v>
+      </c>
+      <c r="G40" s="17" t="s">
+        <v>193</v>
+      </c>
+      <c r="H40" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="D39" s="16" t="s">
-        <v>184</v>
-      </c>
-      <c r="E39" s="16" t="s">
-        <v>185</v>
-      </c>
-      <c r="F39" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="G39" s="16" t="s">
-        <v>187</v>
-      </c>
-      <c r="H39" s="6" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="16">
-        <v>47</v>
-      </c>
-      <c r="B40" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="C40" s="16" t="s">
+    </row>
+    <row r="41" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="17">
+        <v>55</v>
+      </c>
+      <c r="B41" s="17" t="s">
+        <v>172</v>
+      </c>
+      <c r="C41" s="17" t="s">
+        <v>189</v>
+      </c>
+      <c r="D41" s="17" t="s">
+        <v>194</v>
+      </c>
+      <c r="E41" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="F41" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="G41" s="17" t="s">
+        <v>197</v>
+      </c>
+      <c r="H41" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="D40" s="16" t="s">
-        <v>188</v>
-      </c>
-      <c r="E40" s="16" t="s">
+    </row>
+    <row r="42" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="17">
+        <v>56</v>
+      </c>
+      <c r="B42" s="17" t="s">
+        <v>172</v>
+      </c>
+      <c r="C42" s="17" t="s">
         <v>189</v>
       </c>
-      <c r="F40" s="16" t="s">
-        <v>190</v>
-      </c>
-      <c r="G40" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" s="20" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A41" s="16">
-        <v>48</v>
-      </c>
-      <c r="B41" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="C41" s="16" t="s">
-        <v>192</v>
-      </c>
-      <c r="D41" s="16" t="s">
-        <v>193</v>
-      </c>
-      <c r="E41" s="16" t="s">
-        <v>194</v>
-      </c>
-      <c r="F41" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="G41" s="16" t="s">
-        <v>196</v>
-      </c>
-      <c r="H41" s="6" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A42" s="16">
-        <v>49</v>
-      </c>
-      <c r="B42" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="C42" s="16" t="s">
-        <v>192</v>
-      </c>
-      <c r="D42" s="16" t="s">
-        <v>197</v>
-      </c>
-      <c r="E42" s="16" t="s">
+      <c r="D42" s="17" t="s">
         <v>198</v>
       </c>
-      <c r="F42" s="16" t="s">
+      <c r="E42" s="17" t="s">
         <v>199</v>
       </c>
-      <c r="G42" s="16" t="s">
+      <c r="F42" s="17" t="s">
         <v>200</v>
       </c>
-      <c r="H42" s="6" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" s="20" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A43" s="16">
-        <v>50</v>
-      </c>
-      <c r="B43" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="C43" s="16" t="s">
-        <v>192</v>
-      </c>
-      <c r="D43" s="16" t="s">
+      <c r="G42" s="17" t="s">
         <v>201</v>
       </c>
-      <c r="E43" s="16" t="s">
+      <c r="H42" s="7" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="17">
+        <v>57</v>
+      </c>
+      <c r="B43" s="17" t="s">
+        <v>172</v>
+      </c>
+      <c r="C43" s="17" t="s">
         <v>202</v>
       </c>
-      <c r="F43" s="16" t="s">
+      <c r="D43" s="17" t="s">
         <v>203</v>
       </c>
-      <c r="G43" s="16" t="s">
+      <c r="E43" s="17" t="s">
         <v>204</v>
       </c>
-      <c r="H43" s="6" t="s">
-        <v>165</v>
+      <c r="F43" s="17" t="s">
+        <v>205</v>
+      </c>
+      <c r="G43" s="17" t="s">
+        <v>206</v>
+      </c>
+      <c r="H43" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="44" spans="1:8" s="20" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A44" s="17">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B44" s="17" t="s">
-        <v>205</v>
+        <v>172</v>
       </c>
       <c r="C44" s="17" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D44" s="17" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E44" s="17" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F44" s="17" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G44" s="17" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H44" s="7" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="45" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A45" s="17">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B45" s="17" t="s">
-        <v>205</v>
+        <v>172</v>
       </c>
       <c r="C45" s="17" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D45" s="17" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E45" s="17" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F45" s="17" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G45" s="17" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="17">
-        <v>53</v>
-      </c>
-      <c r="B46" s="17" t="s">
-        <v>205</v>
-      </c>
-      <c r="C46" s="17" t="s">
-        <v>206</v>
-      </c>
-      <c r="D46" s="17" t="s">
         <v>217</v>
       </c>
-      <c r="E46" s="17" t="s">
-        <v>218</v>
-      </c>
-      <c r="F46" s="17" t="s">
-        <v>219</v>
-      </c>
-      <c r="G46" s="17" t="s">
-        <v>220</v>
-      </c>
-      <c r="H46" s="7" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A47" s="17">
-        <v>54</v>
-      </c>
-      <c r="B47" s="17" t="s">
-        <v>205</v>
-      </c>
-      <c r="C47" s="17" t="s">
-        <v>222</v>
-      </c>
-      <c r="D47" s="17" t="s">
-        <v>223</v>
-      </c>
-      <c r="E47" s="17" t="s">
-        <v>224</v>
-      </c>
-      <c r="F47" s="17" t="s">
-        <v>225</v>
-      </c>
-      <c r="G47" s="17" t="s">
-        <v>226</v>
-      </c>
-      <c r="H47" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A48" s="17">
-        <v>55</v>
-      </c>
-      <c r="B48" s="17" t="s">
-        <v>205</v>
-      </c>
-      <c r="C48" s="17" t="s">
-        <v>222</v>
-      </c>
-      <c r="D48" s="17" t="s">
-        <v>227</v>
-      </c>
-      <c r="E48" s="17" t="s">
-        <v>228</v>
-      </c>
-      <c r="F48" s="17" t="s">
-        <v>229</v>
-      </c>
-      <c r="G48" s="17" t="s">
-        <v>230</v>
-      </c>
-      <c r="H48" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A49" s="17">
-        <v>56</v>
-      </c>
-      <c r="B49" s="17" t="s">
-        <v>205</v>
-      </c>
-      <c r="C49" s="17" t="s">
-        <v>222</v>
-      </c>
-      <c r="D49" s="17" t="s">
-        <v>231</v>
-      </c>
-      <c r="E49" s="17" t="s">
-        <v>232</v>
-      </c>
-      <c r="F49" s="17" t="s">
-        <v>233</v>
-      </c>
-      <c r="G49" s="17" t="s">
-        <v>234</v>
-      </c>
-      <c r="H49" s="7" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A50" s="17">
-        <v>57</v>
-      </c>
-      <c r="B50" s="17" t="s">
-        <v>205</v>
-      </c>
-      <c r="C50" s="17" t="s">
-        <v>235</v>
-      </c>
-      <c r="D50" s="17" t="s">
-        <v>236</v>
-      </c>
-      <c r="E50" s="17" t="s">
-        <v>237</v>
-      </c>
-      <c r="F50" s="17" t="s">
-        <v>238</v>
-      </c>
-      <c r="G50" s="17" t="s">
-        <v>239</v>
-      </c>
-      <c r="H50" s="7" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" s="20" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A51" s="17">
-        <v>58</v>
-      </c>
-      <c r="B51" s="17" t="s">
-        <v>205</v>
-      </c>
-      <c r="C51" s="17" t="s">
-        <v>235</v>
-      </c>
-      <c r="D51" s="17" t="s">
-        <v>241</v>
-      </c>
-      <c r="E51" s="17" t="s">
-        <v>242</v>
-      </c>
-      <c r="F51" s="17" t="s">
-        <v>243</v>
-      </c>
-      <c r="G51" s="17" t="s">
-        <v>244</v>
-      </c>
-      <c r="H51" s="7" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" s="20" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A52" s="17">
-        <v>59</v>
-      </c>
-      <c r="B52" s="17" t="s">
-        <v>205</v>
-      </c>
-      <c r="C52" s="17" t="s">
-        <v>235</v>
-      </c>
-      <c r="D52" s="17" t="s">
-        <v>246</v>
-      </c>
-      <c r="E52" s="17" t="s">
-        <v>247</v>
-      </c>
-      <c r="F52" s="17" t="s">
-        <v>248</v>
-      </c>
-      <c r="G52" s="17" t="s">
-        <v>249</v>
-      </c>
-      <c r="H52" s="7" t="s">
-        <v>250</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:H52" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A2:H45" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -2894,88 +2851,88 @@
   <sheetData>
     <row r="1" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
-        <v>251</v>
+        <v>218</v>
       </c>
       <c r="B1" s="10"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>252</v>
+        <v>219</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>253</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="66" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
-        <v>254</v>
+        <v>221</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>255</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
-        <v>256</v>
+        <v>223</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>257</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
-        <v>258</v>
+        <v>225</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>259</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
-        <v>260</v>
+        <v>227</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>261</v>
+        <v>228</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
-        <v>262</v>
+        <v>229</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>263</v>
+        <v>230</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>264</v>
+        <v>231</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>265</v>
+        <v>232</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>266</v>
+        <v>233</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>267</v>
+        <v>234</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
-        <v>268</v>
+        <v>235</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>269</v>
+        <v>236</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>270</v>
+        <v>237</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>271</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>